<commit_message>
feat(narrative): add story flow, art, and layout controls
</commit_message>
<xml_diff>
--- a/GameConfig/Datas/Defines/__tables__.xlsx
+++ b/GameConfig/Datas/Defines/__tables__.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2980" yWindow="7260" windowWidth="28800" windowHeight="18470" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="9" customWidth="1" style="4" min="1" max="1"/>
@@ -886,52 +886,176 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>TbReplyOptionConfig</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>ReplyOptionConfig</t>
         </is>
       </c>
-      <c r="D15" t="b">
-        <v>1</v>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D15" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>回复选项配置表.xlsx</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="0" t="inlineStr">
         <is>
           <t>回复选项配置表</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>TbStoryNodeConfig</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>StoryNodeConfig</t>
         </is>
       </c>
-      <c r="D16" t="b">
-        <v>1</v>
-      </c>
-      <c r="E16" t="inlineStr">
+      <c r="D16" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>剧情节点配置表.xlsx</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="0" t="inlineStr">
         <is>
           <t>剧情节点配置表</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="0" t="inlineStr">
+        <is>
+          <t>TbNarrativeSessionConfig</t>
+        </is>
+      </c>
+      <c r="C17" s="0" t="inlineStr">
+        <is>
+          <t>NarrativeSessionConfig</t>
+        </is>
+      </c>
+      <c r="D17" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E17" s="0" t="inlineStr">
+        <is>
+          <t>叙事Session配置表.xlsx</t>
+        </is>
+      </c>
+      <c r="F17" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G17" s="0" t="inlineStr"/>
+      <c r="I17" s="0" t="inlineStr">
+        <is>
+          <t>叙事Session配置表</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="0" t="inlineStr">
+        <is>
+          <t>TbNarrativeActionConfig</t>
+        </is>
+      </c>
+      <c r="C18" s="0" t="inlineStr">
+        <is>
+          <t>NarrativeActionConfig</t>
+        </is>
+      </c>
+      <c r="D18" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E18" s="0" t="inlineStr">
+        <is>
+          <t>叙事动作配置表.xlsx</t>
+        </is>
+      </c>
+      <c r="F18" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G18" s="0" t="inlineStr"/>
+      <c r="I18" s="0" t="inlineStr">
+        <is>
+          <t>叙事动作配置表</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>TbNarrativeItemConfig</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>NarrativeItemConfig</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>叙事物品配置表.xlsx</t>
+        </is>
+      </c>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G19" s="0" t="inlineStr"/>
+      <c r="I19" s="0" t="inlineStr">
+        <is>
+          <t>叙事物品配置表</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>TbNarrativeItemPartConfig</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>NarrativeItemPartConfig</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="b">
+        <v>1</v>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>叙事物品部件配置表.xlsx</t>
+        </is>
+      </c>
+      <c r="F20" s="0" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G20" s="0" t="inlineStr"/>
+      <c r="I20" s="0" t="inlineStr">
+        <is>
+          <t>叙事物品部件配置表</t>
         </is>
       </c>
     </row>

</xml_diff>